<commit_message>
Sync review data 2026-10-01
</commit_message>
<xml_diff>
--- a/review-results/复盘信息抓取-20261001.xlsx
+++ b/review-results/复盘信息抓取-20261001.xlsx
@@ -1125,7 +1125,9 @@
           <t>00:15</t>
         </is>
       </c>
-      <c r="D2" s="3" t="n"/>
+      <c r="D2" s="3" t="n">
+        <v>411.6</v>
+      </c>
       <c r="E2" s="3" t="n">
         <v>441.52</v>
       </c>
@@ -1163,7 +1165,9 @@
           <t>00:30</t>
         </is>
       </c>
-      <c r="D3" s="3" t="n"/>
+      <c r="D3" s="3" t="n">
+        <v>411.6</v>
+      </c>
       <c r="E3" s="3" t="n">
         <v>451.95</v>
       </c>
@@ -1201,7 +1205,9 @@
           <t>00:45</t>
         </is>
       </c>
-      <c r="D4" s="3" t="n"/>
+      <c r="D4" s="3" t="n">
+        <v>411.6</v>
+      </c>
       <c r="E4" s="3" t="n">
         <v>427.86</v>
       </c>
@@ -1239,7 +1245,9 @@
           <t>01:00</t>
         </is>
       </c>
-      <c r="D5" s="3" t="n"/>
+      <c r="D5" s="3" t="n">
+        <v>411.6</v>
+      </c>
       <c r="E5" s="3" t="n">
         <v>425.45</v>
       </c>
@@ -1278,7 +1286,9 @@
           <t>01:15</t>
         </is>
       </c>
-      <c r="D6" s="3" t="n"/>
+      <c r="D6" s="3" t="n">
+        <v>411.6</v>
+      </c>
       <c r="E6" s="3" t="n">
         <v>439.32</v>
       </c>
@@ -1317,7 +1327,9 @@
           <t>01:30</t>
         </is>
       </c>
-      <c r="D7" s="3" t="n"/>
+      <c r="D7" s="3" t="n">
+        <v>411.6</v>
+      </c>
       <c r="E7" s="3" t="n">
         <v>424.63</v>
       </c>
@@ -1356,7 +1368,9 @@
           <t>01:45</t>
         </is>
       </c>
-      <c r="D8" s="3" t="n"/>
+      <c r="D8" s="3" t="n">
+        <v>411.6</v>
+      </c>
       <c r="E8" s="3" t="n">
         <v>409.35</v>
       </c>
@@ -1395,7 +1409,9 @@
           <t>02:00</t>
         </is>
       </c>
-      <c r="D9" s="3" t="n"/>
+      <c r="D9" s="3" t="n">
+        <v>411.6</v>
+      </c>
       <c r="E9" s="3" t="n">
         <v>395</v>
       </c>
@@ -1434,7 +1450,9 @@
           <t>02:15</t>
         </is>
       </c>
-      <c r="D10" s="3" t="n"/>
+      <c r="D10" s="3" t="n">
+        <v>464.17</v>
+      </c>
       <c r="E10" s="3" t="n">
         <v>364.54</v>
       </c>
@@ -1473,7 +1491,9 @@
           <t>02:30</t>
         </is>
       </c>
-      <c r="D11" s="3" t="n"/>
+      <c r="D11" s="3" t="n">
+        <v>464.17</v>
+      </c>
       <c r="E11" s="3" t="n">
         <v>391.75</v>
       </c>
@@ -1512,7 +1532,9 @@
           <t>02:45</t>
         </is>
       </c>
-      <c r="D12" s="3" t="n"/>
+      <c r="D12" s="3" t="n">
+        <v>464.17</v>
+      </c>
       <c r="E12" s="3" t="n">
         <v>375.82</v>
       </c>
@@ -1551,7 +1573,9 @@
           <t>03:00</t>
         </is>
       </c>
-      <c r="D13" s="3" t="n"/>
+      <c r="D13" s="3" t="n">
+        <v>464.17</v>
+      </c>
       <c r="E13" s="3" t="n">
         <v>373.57</v>
       </c>
@@ -1590,7 +1614,9 @@
           <t>03:15</t>
         </is>
       </c>
-      <c r="D14" s="3" t="n"/>
+      <c r="D14" s="3" t="n">
+        <v>385.27</v>
+      </c>
       <c r="E14" s="3" t="n">
         <v>379.3</v>
       </c>
@@ -1628,7 +1654,9 @@
           <t>03:30</t>
         </is>
       </c>
-      <c r="D15" s="3" t="n"/>
+      <c r="D15" s="3" t="n">
+        <v>385.27</v>
+      </c>
       <c r="E15" s="3" t="n">
         <v>382.35</v>
       </c>
@@ -1666,7 +1694,9 @@
           <t>03:45</t>
         </is>
       </c>
-      <c r="D16" s="3" t="n"/>
+      <c r="D16" s="3" t="n">
+        <v>385.27</v>
+      </c>
       <c r="E16" s="3" t="n">
         <v>390.08</v>
       </c>
@@ -1704,7 +1734,9 @@
           <t>04:00</t>
         </is>
       </c>
-      <c r="D17" s="3" t="n"/>
+      <c r="D17" s="3" t="n">
+        <v>385.27</v>
+      </c>
       <c r="E17" s="3" t="n">
         <v>386.75</v>
       </c>
@@ -1742,7 +1774,9 @@
           <t>04:15</t>
         </is>
       </c>
-      <c r="D18" s="3" t="n"/>
+      <c r="D18" s="3" t="n">
+        <v>382.92</v>
+      </c>
       <c r="E18" s="3" t="n">
         <v>380.51</v>
       </c>
@@ -1780,7 +1814,9 @@
           <t>04:30</t>
         </is>
       </c>
-      <c r="D19" s="3" t="n"/>
+      <c r="D19" s="3" t="n">
+        <v>382.92</v>
+      </c>
       <c r="E19" s="3" t="n">
         <v>390.35</v>
       </c>
@@ -1819,7 +1855,9 @@
           <t>04:45</t>
         </is>
       </c>
-      <c r="D20" s="3" t="n"/>
+      <c r="D20" s="3" t="n">
+        <v>382.92</v>
+      </c>
       <c r="E20" s="3" t="n">
         <v>389.14</v>
       </c>
@@ -1858,7 +1896,9 @@
           <t>05:00</t>
         </is>
       </c>
-      <c r="D21" s="3" t="n"/>
+      <c r="D21" s="3" t="n">
+        <v>382.92</v>
+      </c>
       <c r="E21" s="3" t="n">
         <v>383.13</v>
       </c>
@@ -1897,7 +1937,9 @@
           <t>05:15</t>
         </is>
       </c>
-      <c r="D22" s="3" t="n"/>
+      <c r="D22" s="3" t="n">
+        <v>379.75</v>
+      </c>
       <c r="E22" s="3" t="n">
         <v>390.35</v>
       </c>
@@ -1936,7 +1978,9 @@
           <t>05:30</t>
         </is>
       </c>
-      <c r="D23" s="3" t="n"/>
+      <c r="D23" s="3" t="n">
+        <v>379.75</v>
+      </c>
       <c r="E23" s="3" t="n">
         <v>386.8</v>
       </c>
@@ -1975,7 +2019,9 @@
           <t>05:45</t>
         </is>
       </c>
-      <c r="D24" s="3" t="n"/>
+      <c r="D24" s="3" t="n">
+        <v>379.75</v>
+      </c>
       <c r="E24" s="3" t="n">
         <v>390.14</v>
       </c>
@@ -2014,7 +2060,9 @@
           <t>06:00</t>
         </is>
       </c>
-      <c r="D25" s="3" t="n"/>
+      <c r="D25" s="3" t="n">
+        <v>379.75</v>
+      </c>
       <c r="E25" s="3" t="n">
         <v>391.98</v>
       </c>
@@ -2053,7 +2101,9 @@
           <t>06:15</t>
         </is>
       </c>
-      <c r="D26" s="3" t="n"/>
+      <c r="D26" s="3" t="n">
+        <v>382.92</v>
+      </c>
       <c r="E26" s="3" t="n">
         <v>395.82</v>
       </c>
@@ -2092,7 +2142,9 @@
           <t>06:30</t>
         </is>
       </c>
-      <c r="D27" s="3" t="n"/>
+      <c r="D27" s="3" t="n">
+        <v>382.92</v>
+      </c>
       <c r="E27" s="3" t="n">
         <v>385.27</v>
       </c>
@@ -2131,7 +2183,9 @@
           <t>06:45</t>
         </is>
       </c>
-      <c r="D28" s="3" t="n"/>
+      <c r="D28" s="3" t="n">
+        <v>382.92</v>
+      </c>
       <c r="E28" s="3" t="n">
         <v>389.14</v>
       </c>
@@ -2170,7 +2224,9 @@
           <t>07:00</t>
         </is>
       </c>
-      <c r="D29" s="3" t="n"/>
+      <c r="D29" s="3" t="n">
+        <v>382.92</v>
+      </c>
       <c r="E29" s="3" t="n">
         <v>394.72</v>
       </c>
@@ -2209,7 +2265,9 @@
           <t>07:15</t>
         </is>
       </c>
-      <c r="D30" s="3" t="n"/>
+      <c r="D30" s="3" t="n">
+        <v>379.75</v>
+      </c>
       <c r="E30" s="3" t="n">
         <v>432.54</v>
       </c>
@@ -2248,7 +2306,9 @@
           <t>07:30</t>
         </is>
       </c>
-      <c r="D31" s="3" t="n"/>
+      <c r="D31" s="3" t="n">
+        <v>379.75</v>
+      </c>
       <c r="E31" s="3" t="n">
         <v>364.54</v>
       </c>
@@ -2287,7 +2347,9 @@
           <t>07:45</t>
         </is>
       </c>
-      <c r="D32" s="3" t="n"/>
+      <c r="D32" s="3" t="n">
+        <v>379.75</v>
+      </c>
       <c r="E32" s="3" t="n">
         <v>383.52</v>
       </c>
@@ -2326,7 +2388,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="D33" s="3" t="n"/>
+      <c r="D33" s="3" t="n">
+        <v>379.75</v>
+      </c>
       <c r="E33" s="3" t="n">
         <v>356.98</v>
       </c>
@@ -2365,7 +2429,9 @@
           <t>08:15</t>
         </is>
       </c>
-      <c r="D34" s="3" t="n"/>
+      <c r="D34" s="3" t="n">
+        <v>398.42</v>
+      </c>
       <c r="E34" s="3" t="n">
         <v>332.26</v>
       </c>
@@ -2404,7 +2470,9 @@
           <t>08:30</t>
         </is>
       </c>
-      <c r="D35" s="3" t="n"/>
+      <c r="D35" s="3" t="n">
+        <v>398.42</v>
+      </c>
       <c r="E35" s="3" t="n">
         <v>335.41</v>
       </c>
@@ -2443,7 +2511,9 @@
           <t>08:45</t>
         </is>
       </c>
-      <c r="D36" s="3" t="n"/>
+      <c r="D36" s="3" t="n">
+        <v>398.42</v>
+      </c>
       <c r="E36" s="3" t="n">
         <v>0</v>
       </c>
@@ -2482,7 +2552,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="D37" s="3" t="n"/>
+      <c r="D37" s="3" t="n">
+        <v>398.42</v>
+      </c>
       <c r="E37" s="3" t="n">
         <v>0</v>
       </c>
@@ -2521,7 +2593,9 @@
           <t>09:15</t>
         </is>
       </c>
-      <c r="D38" s="3" t="n"/>
+      <c r="D38" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E38" s="3" t="n">
         <v>0</v>
       </c>
@@ -2560,7 +2634,9 @@
           <t>09:30</t>
         </is>
       </c>
-      <c r="D39" s="3" t="n"/>
+      <c r="D39" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E39" s="3" t="n">
         <v>0</v>
       </c>
@@ -2599,7 +2675,9 @@
           <t>09:45</t>
         </is>
       </c>
-      <c r="D40" s="3" t="n"/>
+      <c r="D40" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E40" s="3" t="n">
         <v>0</v>
       </c>
@@ -2638,7 +2716,9 @@
           <t>10:00</t>
         </is>
       </c>
-      <c r="D41" s="3" t="n"/>
+      <c r="D41" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E41" s="3" t="n">
         <v>0</v>
       </c>
@@ -2677,7 +2757,9 @@
           <t>10:15</t>
         </is>
       </c>
-      <c r="D42" s="3" t="n"/>
+      <c r="D42" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E42" s="3" t="n">
         <v>0</v>
       </c>
@@ -2716,7 +2798,9 @@
           <t>10:30</t>
         </is>
       </c>
-      <c r="D43" s="3" t="n"/>
+      <c r="D43" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E43" s="3" t="n">
         <v>0</v>
       </c>
@@ -2755,7 +2839,9 @@
           <t>10:45</t>
         </is>
       </c>
-      <c r="D44" s="3" t="n"/>
+      <c r="D44" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E44" s="3" t="n">
         <v>0</v>
       </c>
@@ -2794,7 +2880,9 @@
           <t>11:00</t>
         </is>
       </c>
-      <c r="D45" s="3" t="n"/>
+      <c r="D45" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E45" s="3" t="n">
         <v>0</v>
       </c>
@@ -2833,7 +2921,9 @@
           <t>11:15</t>
         </is>
       </c>
-      <c r="D46" s="3" t="n"/>
+      <c r="D46" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E46" s="3" t="n">
         <v>0</v>
       </c>
@@ -2872,7 +2962,9 @@
           <t>11:30</t>
         </is>
       </c>
-      <c r="D47" s="3" t="n"/>
+      <c r="D47" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E47" s="3" t="n">
         <v>0</v>
       </c>
@@ -2911,7 +3003,9 @@
           <t>11:45</t>
         </is>
       </c>
-      <c r="D48" s="3" t="n"/>
+      <c r="D48" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E48" s="3" t="n">
         <v>0</v>
       </c>
@@ -2950,7 +3044,9 @@
           <t>12:00</t>
         </is>
       </c>
-      <c r="D49" s="3" t="n"/>
+      <c r="D49" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E49" s="3" t="n">
         <v>0</v>
       </c>
@@ -2989,7 +3085,9 @@
           <t>12:15</t>
         </is>
       </c>
-      <c r="D50" s="3" t="n"/>
+      <c r="D50" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E50" s="3" t="n">
         <v>0</v>
       </c>
@@ -3028,7 +3126,9 @@
           <t>12:30</t>
         </is>
       </c>
-      <c r="D51" s="3" t="n"/>
+      <c r="D51" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E51" s="3" t="n">
         <v>0</v>
       </c>
@@ -3067,7 +3167,9 @@
           <t>12:45</t>
         </is>
       </c>
-      <c r="D52" s="3" t="n"/>
+      <c r="D52" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E52" s="3" t="n">
         <v>0</v>
       </c>
@@ -3106,7 +3208,9 @@
           <t>13:00</t>
         </is>
       </c>
-      <c r="D53" s="3" t="n"/>
+      <c r="D53" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E53" s="3" t="n">
         <v>0</v>
       </c>
@@ -3145,7 +3249,9 @@
           <t>13:15</t>
         </is>
       </c>
-      <c r="D54" s="3" t="n"/>
+      <c r="D54" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E54" s="3" t="n">
         <v>0</v>
       </c>
@@ -3184,7 +3290,9 @@
           <t>13:30</t>
         </is>
       </c>
-      <c r="D55" s="3" t="n"/>
+      <c r="D55" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E55" s="3" t="n">
         <v>0</v>
       </c>
@@ -3223,7 +3331,9 @@
           <t>13:45</t>
         </is>
       </c>
-      <c r="D56" s="3" t="n"/>
+      <c r="D56" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E56" s="3" t="n">
         <v>0</v>
       </c>
@@ -3262,7 +3372,9 @@
           <t>14:00</t>
         </is>
       </c>
-      <c r="D57" s="3" t="n"/>
+      <c r="D57" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E57" s="3" t="n">
         <v>0</v>
       </c>
@@ -3301,7 +3413,9 @@
           <t>14:15</t>
         </is>
       </c>
-      <c r="D58" s="3" t="n"/>
+      <c r="D58" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E58" s="3" t="n">
         <v>0</v>
       </c>
@@ -3340,7 +3454,9 @@
           <t>14:30</t>
         </is>
       </c>
-      <c r="D59" s="3" t="n"/>
+      <c r="D59" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E59" s="3" t="n">
         <v>301.47</v>
       </c>
@@ -3379,7 +3495,9 @@
           <t>14:45</t>
         </is>
       </c>
-      <c r="D60" s="3" t="n"/>
+      <c r="D60" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E60" s="3" t="n">
         <v>331.79</v>
       </c>
@@ -3418,7 +3536,9 @@
           <t>15:00</t>
         </is>
       </c>
-      <c r="D61" s="3" t="n"/>
+      <c r="D61" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E61" s="3" t="n">
         <v>330.26</v>
       </c>
@@ -3457,7 +3577,9 @@
           <t>15:15</t>
         </is>
       </c>
-      <c r="D62" s="3" t="n"/>
+      <c r="D62" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E62" s="3" t="n">
         <v>0</v>
       </c>
@@ -3496,7 +3618,9 @@
           <t>15:30</t>
         </is>
       </c>
-      <c r="D63" s="3" t="n"/>
+      <c r="D63" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E63" s="3" t="n">
         <v>331.79</v>
       </c>
@@ -3535,7 +3659,9 @@
           <t>15:45</t>
         </is>
       </c>
-      <c r="D64" s="3" t="n"/>
+      <c r="D64" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E64" s="3" t="n">
         <v>378.23</v>
       </c>
@@ -3574,7 +3700,9 @@
           <t>16:00</t>
         </is>
       </c>
-      <c r="D65" s="3" t="n"/>
+      <c r="D65" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E65" s="3" t="n">
         <v>359.25</v>
       </c>
@@ -3613,7 +3741,9 @@
           <t>16:15</t>
         </is>
       </c>
-      <c r="D66" s="3" t="n"/>
+      <c r="D66" s="3" t="n">
+        <v>382.91</v>
+      </c>
       <c r="E66" s="3" t="n">
         <v>368.88</v>
       </c>
@@ -3652,7 +3782,9 @@
           <t>16:30</t>
         </is>
       </c>
-      <c r="D67" s="3" t="n"/>
+      <c r="D67" s="3" t="n">
+        <v>382.91</v>
+      </c>
       <c r="E67" s="3" t="n">
         <v>379.3</v>
       </c>
@@ -3691,7 +3823,9 @@
           <t>16:45</t>
         </is>
       </c>
-      <c r="D68" s="3" t="n"/>
+      <c r="D68" s="3" t="n">
+        <v>382.91</v>
+      </c>
       <c r="E68" s="3" t="n">
         <v>400.47</v>
       </c>
@@ -3730,7 +3864,9 @@
           <t>17:00</t>
         </is>
       </c>
-      <c r="D69" s="3" t="n"/>
+      <c r="D69" s="3" t="n">
+        <v>382.91</v>
+      </c>
       <c r="E69" s="3" t="n">
         <v>408.45</v>
       </c>
@@ -3769,7 +3905,9 @@
           <t>17:15</t>
         </is>
       </c>
-      <c r="D70" s="3" t="n"/>
+      <c r="D70" s="3" t="n">
+        <v>368.88</v>
+      </c>
       <c r="E70" s="3" t="n">
         <v>347.32</v>
       </c>
@@ -3808,7 +3946,9 @@
           <t>17:30</t>
         </is>
       </c>
-      <c r="D71" s="3" t="n"/>
+      <c r="D71" s="3" t="n">
+        <v>368.88</v>
+      </c>
       <c r="E71" s="3" t="n">
         <v>395</v>
       </c>
@@ -3847,7 +3987,9 @@
           <t>17:45</t>
         </is>
       </c>
-      <c r="D72" s="3" t="n"/>
+      <c r="D72" s="3" t="n">
+        <v>368.88</v>
+      </c>
       <c r="E72" s="3" t="n">
         <v>393.85</v>
       </c>
@@ -3886,7 +4028,9 @@
           <t>18:00</t>
         </is>
       </c>
-      <c r="D73" s="3" t="n"/>
+      <c r="D73" s="3" t="n">
+        <v>368.88</v>
+      </c>
       <c r="E73" s="3" t="n">
         <v>364.14</v>
       </c>
@@ -3925,7 +4069,9 @@
           <t>18:15</t>
         </is>
       </c>
-      <c r="D74" s="3" t="n"/>
+      <c r="D74" s="3" t="n">
+        <v>454.25</v>
+      </c>
       <c r="E74" s="3" t="n">
         <v>378.75</v>
       </c>
@@ -3964,7 +4110,9 @@
           <t>18:30</t>
         </is>
       </c>
-      <c r="D75" s="3" t="n"/>
+      <c r="D75" s="3" t="n">
+        <v>454.25</v>
+      </c>
       <c r="E75" s="3" t="n">
         <v>364.14</v>
       </c>
@@ -4003,7 +4151,9 @@
           <t>18:45</t>
         </is>
       </c>
-      <c r="D76" s="3" t="n"/>
+      <c r="D76" s="3" t="n">
+        <v>454.25</v>
+      </c>
       <c r="E76" s="3" t="n">
         <v>364.14</v>
       </c>
@@ -4042,7 +4192,9 @@
           <t>19:00</t>
         </is>
       </c>
-      <c r="D77" s="3" t="n"/>
+      <c r="D77" s="3" t="n">
+        <v>454.25</v>
+      </c>
       <c r="E77" s="3" t="n">
         <v>364.14</v>
       </c>
@@ -4081,7 +4233,9 @@
           <t>19:15</t>
         </is>
       </c>
-      <c r="D78" s="3" t="n"/>
+      <c r="D78" s="3" t="n">
+        <v>368.88</v>
+      </c>
       <c r="E78" s="3" t="n">
         <v>364.14</v>
       </c>
@@ -4120,7 +4274,9 @@
           <t>19:30</t>
         </is>
       </c>
-      <c r="D79" s="3" t="n"/>
+      <c r="D79" s="3" t="n">
+        <v>368.88</v>
+      </c>
       <c r="E79" s="3" t="n">
         <v>361.23</v>
       </c>
@@ -4159,7 +4315,9 @@
           <t>19:45</t>
         </is>
       </c>
-      <c r="D80" s="3" t="n"/>
+      <c r="D80" s="3" t="n">
+        <v>368.88</v>
+      </c>
       <c r="E80" s="3" t="n">
         <v>361.23</v>
       </c>
@@ -4198,7 +4356,9 @@
           <t>20:00</t>
         </is>
       </c>
-      <c r="D81" s="3" t="n"/>
+      <c r="D81" s="3" t="n">
+        <v>368.88</v>
+      </c>
       <c r="E81" s="3" t="n">
         <v>364.14</v>
       </c>
@@ -4237,7 +4397,9 @@
           <t>20:15</t>
         </is>
       </c>
-      <c r="D82" s="3" t="n"/>
+      <c r="D82" s="3" t="n">
+        <v>371.85</v>
+      </c>
       <c r="E82" s="3" t="n">
         <v>375.82</v>
       </c>
@@ -4276,7 +4438,9 @@
           <t>20:30</t>
         </is>
       </c>
-      <c r="D83" s="3" t="n"/>
+      <c r="D83" s="3" t="n">
+        <v>371.85</v>
+      </c>
       <c r="E83" s="3" t="n">
         <v>393.85</v>
       </c>
@@ -4315,7 +4479,9 @@
           <t>20:45</t>
         </is>
       </c>
-      <c r="D84" s="3" t="n"/>
+      <c r="D84" s="3" t="n">
+        <v>371.85</v>
+      </c>
       <c r="E84" s="3" t="n">
         <v>427.86</v>
       </c>
@@ -4354,7 +4520,9 @@
           <t>21:00</t>
         </is>
       </c>
-      <c r="D85" s="3" t="n"/>
+      <c r="D85" s="3" t="n">
+        <v>371.85</v>
+      </c>
       <c r="E85" s="3" t="n">
         <v>458.98</v>
       </c>
@@ -4393,7 +4561,9 @@
           <t>21:15</t>
         </is>
       </c>
-      <c r="D86" s="3" t="n"/>
+      <c r="D86" s="3" t="n">
+        <v>371.85</v>
+      </c>
       <c r="E86" s="3" t="n">
         <v>459.86</v>
       </c>
@@ -4432,7 +4602,9 @@
           <t>21:30</t>
         </is>
       </c>
-      <c r="D87" s="3" t="n"/>
+      <c r="D87" s="3" t="n">
+        <v>371.85</v>
+      </c>
       <c r="E87" s="3" t="n">
         <v>457.32</v>
       </c>
@@ -4471,7 +4643,9 @@
           <t>21:45</t>
         </is>
       </c>
-      <c r="D88" s="3" t="n"/>
+      <c r="D88" s="3" t="n">
+        <v>371.85</v>
+      </c>
       <c r="E88" s="3" t="n">
         <v>443.19</v>
       </c>
@@ -4510,7 +4684,9 @@
           <t>22:00</t>
         </is>
       </c>
-      <c r="D89" s="3" t="n"/>
+      <c r="D89" s="3" t="n">
+        <v>371.85</v>
+      </c>
       <c r="E89" s="3" t="n">
         <v>426.77</v>
       </c>
@@ -4549,7 +4725,9 @@
           <t>22:15</t>
         </is>
       </c>
-      <c r="D90" s="3" t="n"/>
+      <c r="D90" s="3" t="n">
+        <v>371.85</v>
+      </c>
       <c r="E90" s="3" t="n">
         <v>414.76</v>
       </c>
@@ -4588,7 +4766,9 @@
           <t>22:30</t>
         </is>
       </c>
-      <c r="D91" s="3" t="n"/>
+      <c r="D91" s="3" t="n">
+        <v>371.85</v>
+      </c>
       <c r="E91" s="3" t="n">
         <v>411.6</v>
       </c>
@@ -4627,7 +4807,9 @@
           <t>22:45</t>
         </is>
       </c>
-      <c r="D92" s="3" t="n"/>
+      <c r="D92" s="3" t="n">
+        <v>371.85</v>
+      </c>
       <c r="E92" s="3" t="n">
         <v>414.76</v>
       </c>
@@ -4666,7 +4848,9 @@
           <t>23:00</t>
         </is>
       </c>
-      <c r="D93" s="3" t="n"/>
+      <c r="D93" s="3" t="n">
+        <v>371.85</v>
+      </c>
       <c r="E93" s="3" t="n">
         <v>451.95</v>
       </c>
@@ -4704,7 +4888,9 @@
           <t>23:15</t>
         </is>
       </c>
-      <c r="D94" s="3" t="n"/>
+      <c r="D94" s="3" t="n">
+        <v>368.88</v>
+      </c>
       <c r="E94" s="3" t="n">
         <v>458.98</v>
       </c>
@@ -4742,7 +4928,9 @@
           <t>23:30</t>
         </is>
       </c>
-      <c r="D95" s="3" t="n"/>
+      <c r="D95" s="3" t="n">
+        <v>368.88</v>
+      </c>
       <c r="E95" s="3" t="n">
         <v>458.98</v>
       </c>
@@ -4780,7 +4968,9 @@
           <t>23:45</t>
         </is>
       </c>
-      <c r="D96" s="3" t="n"/>
+      <c r="D96" s="3" t="n">
+        <v>368.88</v>
+      </c>
       <c r="E96" s="3" t="n">
         <v>456.97</v>
       </c>
@@ -4818,7 +5008,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="D97" s="3" t="n"/>
+      <c r="D97" s="3" t="n">
+        <v>368.88</v>
+      </c>
       <c r="E97" s="3" t="n">
         <v>459.54</v>
       </c>
@@ -17206,7 +17398,7 @@
         <v>96</v>
       </c>
       <c r="C10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">

</xml_diff>